<commit_message>
test(hrm): payroll samples for severance and job-loss allowances
C18 (mutual agreement, 1.5 years on a 22,000,000 average) and C19
(restructuring, the two-month floor), with the allowance in a new
column AI after the notes; the 28 existing rows keep their figures.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/payroll-samples/payroll-input-samples.xlsx
+++ b/docs/payroll-samples/payroll-input-samples.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="237">
   <si>
     <t>Mã</t>
   </si>
@@ -118,6 +118,9 @@
     <t>Nguồn số liệu</t>
   </si>
   <si>
+    <t>Trợ cấp thôi việc/mất việc</t>
+  </si>
+  <si>
     <t>S01</t>
   </si>
   <si>
@@ -406,6 +409,36 @@
     <t>40 giờ đầu miễn thuế, 4 giờ vượt giới hạn chịu thuế. Hệ thống phải cảnh báo khi vượt</t>
   </si>
   <si>
+    <t>C18</t>
+  </si>
+  <si>
+    <t>Nghỉ việc theo thỏa thuận, có trợ cấp thôi việc</t>
+  </si>
+  <si>
+    <t>Vào làm 01/07/2007, ngày làm cuối 15/04/2026 (thỏa thuận chấm dứt). Lương 20.000.000, phụ lục 24.000.000 từ 01/01/2026. Tham gia BHTN từ 01/01/2009: 207 tháng. Công hưởng lương 11</t>
+  </si>
+  <si>
+    <t>Thời gian làm việc 225 tháng − 207 tháng đóng BHTN = 18 tháng = 1,5 năm (tháng lẻ ≤ 6 tính 1/2 năm, khoản 3 Điều 8 NĐ 145/2020). Lương bình quân 6 tháng liền kề 10/2025–03/2026 = 22.000.000 (khoản 5 Điều 8 NĐ 145/2020). Trợ cấp = 1,5 × 1/2 × 22.000.000 (Điều 46 BLLĐ 2019); không tính BH, không chịu thuế TNCN</t>
+  </si>
+  <si>
+    <t>thuế, BH người lao động và doanh nghiệp: khớp thue-2026; thuế khớp pit; chia lương theo công, phép chưa nghỉ: tự tính; trợ cấp thôi việc/mất việc: tự tính</t>
+  </si>
+  <si>
+    <t>C19</t>
+  </si>
+  <si>
+    <t>Cho thôi việc do cơ cấu lại, trợ cấp mất việc tối thiểu</t>
+  </si>
+  <si>
+    <t>Vào làm 01/03/2024, ngày làm cuối 30/04/2026 (cơ cấu lại, Điều 42 BLLĐ 2019). Đóng BHTN cả 26 tháng</t>
+  </si>
+  <si>
+    <t>Thời gian tính trợ cấp 26 − 26 = 0 năm, nhưng trợ cấp mất việc ít nhất 2 tháng lương: 2 × 15.000.000 (Điều 47 BLLĐ 2019); không tính BH, không chịu thuế TNCN</t>
+  </si>
+  <si>
+    <t>thuế, BH người lao động và doanh nghiệp: khớp thue-2026; thuế khớp pit; trợ cấp thôi việc/mất việc: tự tính</t>
+  </si>
+  <si>
     <t>#</t>
   </si>
   <si>
@@ -493,6 +526,15 @@
     <t>Khoản 3 Điều 113 BLLĐ 2019; Điều 67 NĐ 145/2020; khoản 8 Điều 4 Luật 109/2025 (Bộ Tài chính trả lời: gồm cả phép chưa nghỉ khi thôi việc)</t>
   </si>
   <si>
+    <t>Trợ cấp thôi việc, mất việc</t>
+  </si>
+  <si>
+    <t>Thời gian tính = số tháng làm việc (bỏ ngày lẻ) − số tháng đóng BHTN − số tháng đã chi trợ cấp; tháng lẻ ≤ 6 tính 1/2 năm, &gt; 6 tính 1 năm; làm đủ 12 tháng mới hưởng. Lương bình quân = lương + phụ cấp lương của hợp đồng hiệu lực cuối mỗi tháng trong 6 tháng liền trước tháng nghỉ việc. Thôi việc 1/2 tháng mỗi năm; mất việc 1 tháng mỗi năm, ít nhất 2 tháng. Trả ở bảng lương tháng nghỉ việc; không tính BH, không chịu thuế TNCN.</t>
+  </si>
+  <si>
+    <t>Điều 46, 47, 48 BLLĐ 2019; khoản 3, 5 Điều 8 NĐ 145/2020; không tính vào thu nhập chịu thuế từ tiền lương (điểm b khoản 2 Điều 2 TT 111/2013/TT-BTC; Luật Thuế TNCN 109/2025/QH15, CẦN kế toán xác nhận điều khoản). Bỏ ngày lẻ và cách lấy 6 tháng là giả định</t>
+  </si>
+  <si>
     <t>Lương hợp đồng + phụ cấp lương, không chia theo công. Đổi lương giữa tháng: lấy mức hiệu lực cuối tháng.</t>
   </si>
   <si>
@@ -565,7 +607,7 @@
     <t>Chưa có trong mẫu</t>
   </si>
   <si>
-    <t>Đoàn phí công đoàn của người lao động, khoản hỗ trợ miễn thuế (ăn ca…), người không cư trú, HĐ dưới 3 tháng, truy thu khác năm, vượt giới hạn tăng ca năm.</t>
+    <t>Trợ cấp thôi việc khi nhập muộn sau kỳ đã chốt, đoàn phí công đoàn của người lao động, khoản hỗ trợ miễn thuế (ăn ca…), người không cư trú, HĐ dưới 3 tháng, truy thu khác năm, vượt giới hạn tăng ca năm.</t>
   </si>
   <si>
     <t>Bổ sung khi cần</t>
@@ -1074,7 +1116,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AH29"/>
+  <dimension ref="A1:AI31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1100,9 +1142,10 @@
     <col min="32" max="32" width="15" style="1" customWidth="1"/>
     <col min="33" max="33" width="48" style="2" customWidth="1"/>
     <col min="34" max="34" width="40" customWidth="1"/>
+    <col min="35" max="35" width="14" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1205,16 +1248,19 @@
       <c r="AH1" s="3" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI1" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D2" s="1">
         <v>8000000</v>
@@ -1226,7 +1272,7 @@
         <v>0</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -1259,11 +1305,11 @@
         <v>0</v>
       </c>
       <c r="Q2" s="1">
-        <f>K2+N2+O2+P2</f>
+        <f>K2+N2+O2+P2+AI2</f>
         <v>8000000</v>
       </c>
       <c r="R2" s="1">
-        <f>ROUND((D2+E2)/I2/8*M2*MIN(L2,40),0)+O2</f>
+        <f>ROUND((D2+E2)/I2/8*M2*MIN(L2,40),0)+O2+AI2</f>
         <v>0</v>
       </c>
       <c r="S2" s="1">
@@ -1311,21 +1357,24 @@
         <v>9880000</v>
       </c>
       <c r="AG2" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AH2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="AI2" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D3" s="1">
         <v>18000000</v>
@@ -1337,7 +1386,7 @@
         <v>0</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -1370,11 +1419,11 @@
         <v>0</v>
       </c>
       <c r="Q3" s="1">
-        <f>K3+N3+O3+P3</f>
+        <f>K3+N3+O3+P3+AI3</f>
         <v>18000000</v>
       </c>
       <c r="R3" s="1">
-        <f>ROUND((D3+E3)/I3/8*M3*MIN(L3,40),0)+O3</f>
+        <f>ROUND((D3+E3)/I3/8*M3*MIN(L3,40),0)+O3+AI3</f>
         <v>0</v>
       </c>
       <c r="S3" s="1">
@@ -1422,21 +1471,24 @@
         <v>22230000</v>
       </c>
       <c r="AG3" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AH3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:34" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="AI3" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D4" s="1">
         <v>30000000</v>
@@ -1448,7 +1500,7 @@
         <v>0</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -1481,11 +1533,11 @@
         <v>0</v>
       </c>
       <c r="Q4" s="1">
-        <f>K4+N4+O4+P4</f>
+        <f>K4+N4+O4+P4+AI4</f>
         <v>30000000</v>
       </c>
       <c r="R4" s="1">
-        <f>ROUND((D4+E4)/I4/8*M4*MIN(L4,40),0)+O4</f>
+        <f>ROUND((D4+E4)/I4/8*M4*MIN(L4,40),0)+O4+AI4</f>
         <v>0</v>
       </c>
       <c r="S4" s="1">
@@ -1533,21 +1585,24 @@
         <v>37050000</v>
       </c>
       <c r="AG4" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AH4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="5" spans="1:34" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="AI4" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D5" s="1">
         <v>30000000</v>
@@ -1559,7 +1614,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H5">
         <v>2</v>
@@ -1592,11 +1647,11 @@
         <v>0</v>
       </c>
       <c r="Q5" s="1">
-        <f>K5+N5+O5+P5</f>
+        <f>K5+N5+O5+P5+AI5</f>
         <v>30000000</v>
       </c>
       <c r="R5" s="1">
-        <f>ROUND((D5+E5)/I5/8*M5*MIN(L5,40),0)+O5</f>
+        <f>ROUND((D5+E5)/I5/8*M5*MIN(L5,40),0)+O5+AI5</f>
         <v>0</v>
       </c>
       <c r="S5" s="1">
@@ -1644,21 +1699,24 @@
         <v>37050000</v>
       </c>
       <c r="AG5" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AH5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:34" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="AI5" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D6" s="1">
         <v>45000000</v>
@@ -1670,7 +1728,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H6">
         <v>1</v>
@@ -1703,11 +1761,11 @@
         <v>0</v>
       </c>
       <c r="Q6" s="1">
-        <f>K6+N6+O6+P6</f>
+        <f>K6+N6+O6+P6+AI6</f>
         <v>45000000</v>
       </c>
       <c r="R6" s="1">
-        <f>ROUND((D6+E6)/I6/8*M6*MIN(L6,40),0)+O6</f>
+        <f>ROUND((D6+E6)/I6/8*M6*MIN(L6,40),0)+O6+AI6</f>
         <v>0</v>
       </c>
       <c r="S6" s="1">
@@ -1755,21 +1813,24 @@
         <v>55575000</v>
       </c>
       <c r="AG6" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AH6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:34" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="AI6" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D7" s="1">
         <v>55000000</v>
@@ -1781,7 +1842,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -1814,11 +1875,11 @@
         <v>0</v>
       </c>
       <c r="Q7" s="1">
-        <f>K7+N7+O7+P7</f>
+        <f>K7+N7+O7+P7+AI7</f>
         <v>55000000</v>
       </c>
       <c r="R7" s="1">
-        <f>ROUND((D7+E7)/I7/8*M7*MIN(L7,40),0)+O7</f>
+        <f>ROUND((D7+E7)/I7/8*M7*MIN(L7,40),0)+O7+AI7</f>
         <v>0</v>
       </c>
       <c r="S7" s="1">
@@ -1866,21 +1927,24 @@
         <v>66080000</v>
       </c>
       <c r="AG7" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AH7" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="8" spans="1:34" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="AI7" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D8" s="1">
         <v>90000000</v>
@@ -1892,7 +1956,7 @@
         <v>0</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -1925,11 +1989,11 @@
         <v>0</v>
       </c>
       <c r="Q8" s="1">
-        <f>K8+N8+O8+P8</f>
+        <f>K8+N8+O8+P8+AI8</f>
         <v>90000000</v>
       </c>
       <c r="R8" s="1">
-        <f>ROUND((D8+E8)/I8/8*M8*MIN(L8,40),0)+O8</f>
+        <f>ROUND((D8+E8)/I8/8*M8*MIN(L8,40),0)+O8+AI8</f>
         <v>0</v>
       </c>
       <c r="S8" s="1">
@@ -1977,21 +2041,24 @@
         <v>101430000</v>
       </c>
       <c r="AG8" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AH8" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="9" spans="1:34" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="AI8" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D9" s="1">
         <v>120000000</v>
@@ -2003,7 +2070,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H9">
         <v>0</v>
@@ -2036,11 +2103,11 @@
         <v>0</v>
       </c>
       <c r="Q9" s="1">
-        <f>K9+N9+O9+P9</f>
+        <f>K9+N9+O9+P9+AI9</f>
         <v>120000000</v>
       </c>
       <c r="R9" s="1">
-        <f>ROUND((D9+E9)/I9/8*M9*MIN(L9,40),0)+O9</f>
+        <f>ROUND((D9+E9)/I9/8*M9*MIN(L9,40),0)+O9+AI9</f>
         <v>0</v>
       </c>
       <c r="S9" s="1">
@@ -2088,21 +2155,24 @@
         <v>131592000</v>
       </c>
       <c r="AG9" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AH9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="10" spans="1:34" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="AI9" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D10" s="1">
         <v>150000000</v>
@@ -2114,7 +2184,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H10">
         <v>3</v>
@@ -2147,11 +2217,11 @@
         <v>0</v>
       </c>
       <c r="Q10" s="1">
-        <f>K10+N10+O10+P10</f>
+        <f>K10+N10+O10+P10+AI10</f>
         <v>150000000</v>
       </c>
       <c r="R10" s="1">
-        <f>ROUND((D10+E10)/I10/8*M10*MIN(L10,40),0)+O10</f>
+        <f>ROUND((D10+E10)/I10/8*M10*MIN(L10,40),0)+O10+AI10</f>
         <v>0</v>
       </c>
       <c r="S10" s="1">
@@ -2199,21 +2269,24 @@
         <v>161592000</v>
       </c>
       <c r="AG10" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AH10" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="11" spans="1:34" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="AI10" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D11" s="1">
         <v>22000000</v>
@@ -2225,7 +2298,7 @@
         <v>8000000</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H11">
         <v>0</v>
@@ -2258,11 +2331,11 @@
         <v>0</v>
       </c>
       <c r="Q11" s="1">
-        <f>K11+N11+O11+P11</f>
+        <f>K11+N11+O11+P11+AI11</f>
         <v>30000000</v>
       </c>
       <c r="R11" s="1">
-        <f>ROUND((D11+E11)/I11/8*M11*MIN(L11,40),0)+O11</f>
+        <f>ROUND((D11+E11)/I11/8*M11*MIN(L11,40),0)+O11+AI11</f>
         <v>0</v>
       </c>
       <c r="S11" s="1">
@@ -2310,21 +2383,24 @@
         <v>35170000</v>
       </c>
       <c r="AG11" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="AH11" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="12" spans="1:34" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="AI11" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D12" s="1">
         <v>22000000</v>
@@ -2336,7 +2412,7 @@
         <v>0</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H12">
         <v>1</v>
@@ -2369,11 +2445,11 @@
         <v>0</v>
       </c>
       <c r="Q12" s="1">
-        <f>K12+N12+O12+P12</f>
+        <f>K12+N12+O12+P12+AI12</f>
         <v>25000000</v>
       </c>
       <c r="R12" s="1">
-        <f>ROUND((D12+E12)/I12/8*M12*MIN(L12,40),0)+O12</f>
+        <f>ROUND((D12+E12)/I12/8*M12*MIN(L12,40),0)+O12+AI12</f>
         <v>0</v>
       </c>
       <c r="S12" s="1">
@@ -2421,21 +2497,24 @@
         <v>30875000</v>
       </c>
       <c r="AG12" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="AH12" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="13" spans="1:34" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="AI12" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D13" s="1">
         <v>20000000</v>
@@ -2447,7 +2526,7 @@
         <v>0</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H13">
         <v>0</v>
@@ -2480,11 +2559,11 @@
         <v>0</v>
       </c>
       <c r="Q13" s="1">
-        <f>K13+N13+O13+P13</f>
+        <f>K13+N13+O13+P13+AI13</f>
         <v>10000000</v>
       </c>
       <c r="R13" s="1">
-        <f>ROUND((D13+E13)/I13/8*M13*MIN(L13,40),0)+O13</f>
+        <f>ROUND((D13+E13)/I13/8*M13*MIN(L13,40),0)+O13+AI13</f>
         <v>0</v>
       </c>
       <c r="S13" s="1">
@@ -2532,21 +2611,24 @@
         <v>14700000</v>
       </c>
       <c r="AG13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="AH13" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="14" spans="1:34" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="AI13" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C14" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D14" s="1">
         <v>20000000</v>
@@ -2558,7 +2640,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H14">
         <v>0</v>
@@ -2591,11 +2673,11 @@
         <v>0</v>
       </c>
       <c r="Q14" s="1">
-        <f>K14+N14+O14+P14</f>
+        <f>K14+N14+O14+P14+AI14</f>
         <v>6363636</v>
       </c>
       <c r="R14" s="1">
-        <f>ROUND((D14+E14)/I14/8*M14*MIN(L14,40),0)+O14</f>
+        <f>ROUND((D14+E14)/I14/8*M14*MIN(L14,40),0)+O14+AI14</f>
         <v>0</v>
       </c>
       <c r="S14" s="1">
@@ -2643,21 +2725,24 @@
         <v>6363636</v>
       </c>
       <c r="AG14" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AH14" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="15" spans="1:34" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="AI14" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B15" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C15" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D15" s="1">
         <v>18000000</v>
@@ -2669,7 +2754,7 @@
         <v>0</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H15">
         <v>0</v>
@@ -2702,11 +2787,11 @@
         <v>0</v>
       </c>
       <c r="Q15" s="1">
-        <f>K15+N15+O15+P15</f>
+        <f>K15+N15+O15+P15+AI15</f>
         <v>9818182</v>
       </c>
       <c r="R15" s="1">
-        <f>ROUND((D15+E15)/I15/8*M15*MIN(L15,40),0)+O15</f>
+        <f>ROUND((D15+E15)/I15/8*M15*MIN(L15,40),0)+O15+AI15</f>
         <v>3272727</v>
       </c>
       <c r="S15" s="1">
@@ -2754,21 +2839,24 @@
         <v>9818182</v>
       </c>
       <c r="AG15" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="AH15" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="16" spans="1:34" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="AI15" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C16" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D16" s="1">
         <v>25000000</v>
@@ -2780,7 +2868,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H16">
         <v>0</v>
@@ -2813,11 +2901,11 @@
         <v>0</v>
       </c>
       <c r="Q16" s="1">
-        <f>K16+N16+O16+P16</f>
+        <f>K16+N16+O16+P16+AI16</f>
         <v>22500000</v>
       </c>
       <c r="R16" s="1">
-        <f>ROUND((D16+E16)/I16/8*M16*MIN(L16,40),0)+O16</f>
+        <f>ROUND((D16+E16)/I16/8*M16*MIN(L16,40),0)+O16+AI16</f>
         <v>0</v>
       </c>
       <c r="S16" s="1">
@@ -2865,21 +2953,24 @@
         <v>28375000</v>
       </c>
       <c r="AG16" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="AH16" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="17" spans="1:34" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="AI16" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B17" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D17" s="1">
         <v>25000000</v>
@@ -2891,7 +2982,7 @@
         <v>0</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H17">
         <v>0</v>
@@ -2924,11 +3015,11 @@
         <v>0</v>
       </c>
       <c r="Q17" s="1">
-        <f>K17+N17+O17+P17</f>
+        <f>K17+N17+O17+P17+AI17</f>
         <v>21590909</v>
       </c>
       <c r="R17" s="1">
-        <f>ROUND((D17+E17)/I17/8*M17*MIN(L17,40),0)+O17</f>
+        <f>ROUND((D17+E17)/I17/8*M17*MIN(L17,40),0)+O17+AI17</f>
         <v>0</v>
       </c>
       <c r="S17" s="1">
@@ -2976,21 +3067,24 @@
         <v>27465909</v>
       </c>
       <c r="AG17" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AH17" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="18" spans="1:34" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="AI17" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B18" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C18" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D18" s="1">
         <v>25000000</v>
@@ -3002,7 +3096,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H18">
         <v>0</v>
@@ -3035,11 +3129,11 @@
         <v>0</v>
       </c>
       <c r="Q18" s="1">
-        <f>K18+N18+O18+P18</f>
+        <f>K18+N18+O18+P18+AI18</f>
         <v>19318182</v>
       </c>
       <c r="R18" s="1">
-        <f>ROUND((D18+E18)/I18/8*M18*MIN(L18,40),0)+O18</f>
+        <f>ROUND((D18+E18)/I18/8*M18*MIN(L18,40),0)+O18+AI18</f>
         <v>0</v>
       </c>
       <c r="S18" s="1">
@@ -3087,21 +3181,24 @@
         <v>25193182</v>
       </c>
       <c r="AG18" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AH18" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="19" spans="1:34" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="AI18" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B19" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C19" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D19" s="1">
         <v>25000000</v>
@@ -3113,7 +3210,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H19">
         <v>0</v>
@@ -3146,11 +3243,11 @@
         <v>0</v>
       </c>
       <c r="Q19" s="1">
-        <f>K19+N19+O19+P19</f>
+        <f>K19+N19+O19+P19+AI19</f>
         <v>25000000</v>
       </c>
       <c r="R19" s="1">
-        <f>ROUND((D19+E19)/I19/8*M19*MIN(L19,40),0)+O19</f>
+        <f>ROUND((D19+E19)/I19/8*M19*MIN(L19,40),0)+O19+AI19</f>
         <v>0</v>
       </c>
       <c r="S19" s="1">
@@ -3198,21 +3295,24 @@
         <v>30875000</v>
       </c>
       <c r="AG19" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="AH19" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="20" spans="1:34" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="AI19" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B20" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C20" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D20" s="1">
         <v>20000000</v>
@@ -3224,7 +3324,7 @@
         <v>0</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H20">
         <v>0</v>
@@ -3257,11 +3357,11 @@
         <v>0</v>
       </c>
       <c r="Q20" s="1">
-        <f>K20+N20+O20+P20</f>
+        <f>K20+N20+O20+P20+AI20</f>
         <v>21704545</v>
       </c>
       <c r="R20" s="1">
-        <f>ROUND((D20+E20)/I20/8*M20*MIN(L20,40),0)+O20</f>
+        <f>ROUND((D20+E20)/I20/8*M20*MIN(L20,40),0)+O20+AI20</f>
         <v>1704545</v>
       </c>
       <c r="S20" s="1">
@@ -3309,21 +3409,24 @@
         <v>26404545</v>
       </c>
       <c r="AG20" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AH20" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="21" spans="1:34" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+      <c r="AI20" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B21" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C21" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D21" s="1">
         <v>20000000</v>
@@ -3335,7 +3438,7 @@
         <v>0</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H21">
         <v>0</v>
@@ -3368,11 +3471,11 @@
         <v>0</v>
       </c>
       <c r="Q21" s="1">
-        <f>K21+N21+O21+P21</f>
+        <f>K21+N21+O21+P21+AI21</f>
         <v>21818182</v>
       </c>
       <c r="R21" s="1">
-        <f>ROUND((D21+E21)/I21/8*M21*MIN(L21,40),0)+O21</f>
+        <f>ROUND((D21+E21)/I21/8*M21*MIN(L21,40),0)+O21+AI21</f>
         <v>1818182</v>
       </c>
       <c r="S21" s="1">
@@ -3420,21 +3523,24 @@
         <v>26518182</v>
       </c>
       <c r="AG21" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AH21" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="22" spans="1:34" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+      <c r="AI21" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B22" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D22" s="1">
         <v>20000000</v>
@@ -3446,7 +3552,7 @@
         <v>0</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H22">
         <v>0</v>
@@ -3479,11 +3585,11 @@
         <v>0</v>
       </c>
       <c r="Q22" s="1">
-        <f>K22+N22+O22+P22</f>
+        <f>K22+N22+O22+P22+AI22</f>
         <v>22727273</v>
       </c>
       <c r="R22" s="1">
-        <f>ROUND((D22+E22)/I22/8*M22*MIN(L22,40),0)+O22</f>
+        <f>ROUND((D22+E22)/I22/8*M22*MIN(L22,40),0)+O22+AI22</f>
         <v>2727273</v>
       </c>
       <c r="S22" s="1">
@@ -3531,21 +3637,24 @@
         <v>27427273</v>
       </c>
       <c r="AG22" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AH22" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="23" spans="1:34" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+      <c r="AI22" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B23" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C23" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D23" s="1">
         <v>20000000</v>
@@ -3557,7 +3666,7 @@
         <v>0</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H23">
         <v>0</v>
@@ -3590,11 +3699,11 @@
         <v>0</v>
       </c>
       <c r="Q23" s="1">
-        <f>K23+N23+O23+P23</f>
+        <f>K23+N23+O23+P23+AI23</f>
         <v>20909091</v>
       </c>
       <c r="R23" s="1">
-        <f>ROUND((D23+E23)/I23/8*M23*MIN(L23,40),0)+O23</f>
+        <f>ROUND((D23+E23)/I23/8*M23*MIN(L23,40),0)+O23+AI23</f>
         <v>909091</v>
       </c>
       <c r="S23" s="1">
@@ -3642,21 +3751,24 @@
         <v>25609091</v>
       </c>
       <c r="AG23" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AH23" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="24" spans="1:34" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+      <c r="AI23" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B24" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C24" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D24" s="1">
         <v>60000000</v>
@@ -3668,7 +3780,7 @@
         <v>0</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H24">
         <v>2</v>
@@ -3701,11 +3813,11 @@
         <v>0</v>
       </c>
       <c r="Q24" s="1">
-        <f>K24+N24+O24+P24</f>
+        <f>K24+N24+O24+P24+AI24</f>
         <v>66136364</v>
       </c>
       <c r="R24" s="1">
-        <f>ROUND((D24+E24)/I24/8*M24*MIN(L24,40),0)+O24</f>
+        <f>ROUND((D24+E24)/I24/8*M24*MIN(L24,40),0)+O24+AI24</f>
         <v>6136364</v>
       </c>
       <c r="S24" s="1">
@@ -3753,21 +3865,24 @@
         <v>77266364</v>
       </c>
       <c r="AG24" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AH24" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="25" spans="1:34" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+      <c r="AI24" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B25" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C25" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D25" s="1">
         <v>30000000</v>
@@ -3779,7 +3894,7 @@
         <v>0</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H25">
         <v>0</v>
@@ -3812,11 +3927,11 @@
         <v>2000000</v>
       </c>
       <c r="Q25" s="1">
-        <f>K25+N25+O25+P25</f>
+        <f>K25+N25+O25+P25+AI25</f>
         <v>32000000</v>
       </c>
       <c r="R25" s="1">
-        <f>ROUND((D25+E25)/I25/8*M25*MIN(L25,40),0)+O25</f>
+        <f>ROUND((D25+E25)/I25/8*M25*MIN(L25,40),0)+O25+AI25</f>
         <v>0</v>
       </c>
       <c r="S25" s="1">
@@ -3864,21 +3979,24 @@
         <v>39050000</v>
       </c>
       <c r="AG25" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="AH25" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="26" spans="1:34" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="AI25" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B26" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C26" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D26" s="1">
         <v>30000000</v>
@@ -3890,7 +4008,7 @@
         <v>0</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H26">
         <v>0</v>
@@ -3923,11 +4041,11 @@
         <v>-1500000</v>
       </c>
       <c r="Q26" s="1">
-        <f>K26+N26+O26+P26</f>
+        <f>K26+N26+O26+P26+AI26</f>
         <v>28500000</v>
       </c>
       <c r="R26" s="1">
-        <f>ROUND((D26+E26)/I26/8*M26*MIN(L26,40),0)+O26</f>
+        <f>ROUND((D26+E26)/I26/8*M26*MIN(L26,40),0)+O26+AI26</f>
         <v>0</v>
       </c>
       <c r="S26" s="1">
@@ -3975,21 +4093,24 @@
         <v>35550000</v>
       </c>
       <c r="AG26" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH26" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="27" spans="1:34" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="AI26" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B27" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C27" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D27" s="1">
         <v>60000000</v>
@@ -4001,7 +4122,7 @@
         <v>0</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H27">
         <v>0</v>
@@ -4034,11 +4155,11 @@
         <v>0</v>
       </c>
       <c r="Q27" s="1">
-        <f>K27+N27+O27+P27</f>
+        <f>K27+N27+O27+P27+AI27</f>
         <v>60000000</v>
       </c>
       <c r="R27" s="1">
-        <f>ROUND((D27+E27)/I27/8*M27*MIN(L27,40),0)+O27</f>
+        <f>ROUND((D27+E27)/I27/8*M27*MIN(L27,40),0)+O27+AI27</f>
         <v>0</v>
       </c>
       <c r="S27" s="1">
@@ -4086,21 +4207,24 @@
         <v>71985000</v>
       </c>
       <c r="AG27" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AH27" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="28" spans="1:34" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="AI27" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B28" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C28" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D28" s="1">
         <v>20000000</v>
@@ -4112,7 +4236,7 @@
         <v>0</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H28">
         <v>0</v>
@@ -4145,11 +4269,11 @@
         <v>0</v>
       </c>
       <c r="Q28" s="1">
-        <f>K28+N28+O28+P28</f>
+        <f>K28+N28+O28+P28+AI28</f>
         <v>24960227</v>
       </c>
       <c r="R28" s="1">
-        <f>ROUND((D28+E28)/I28/8*M28*MIN(L28,40),0)+O28</f>
+        <f>ROUND((D28+E28)/I28/8*M28*MIN(L28,40),0)+O28+AI28</f>
         <v>1960227</v>
       </c>
       <c r="S28" s="1">
@@ -4197,21 +4321,24 @@
         <v>30365227</v>
       </c>
       <c r="AG28" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="AH28" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="29" spans="1:34" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+      <c r="AI28" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B29" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C29" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D29" s="1">
         <v>20000000</v>
@@ -4223,7 +4350,7 @@
         <v>0</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H29">
         <v>0</v>
@@ -4256,11 +4383,11 @@
         <v>0</v>
       </c>
       <c r="Q29" s="1">
-        <f>K29+N29+O29+P29</f>
+        <f>K29+N29+O29+P29+AI29</f>
         <v>27500000</v>
       </c>
       <c r="R29" s="1">
-        <f>ROUND((D29+E29)/I29/8*M29*MIN(L29,40),0)+O29</f>
+        <f>ROUND((D29+E29)/I29/8*M29*MIN(L29,40),0)+O29+AI29</f>
         <v>6818182</v>
       </c>
       <c r="S29" s="1">
@@ -4308,10 +4435,241 @@
         <v>32200000</v>
       </c>
       <c r="AG29" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="AH29" t="s">
-        <v>95</v>
+        <v>96</v>
+      </c>
+      <c r="AI29" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>131</v>
+      </c>
+      <c r="B30" t="s">
+        <v>132</v>
+      </c>
+      <c r="C30" t="s">
+        <v>37</v>
+      </c>
+      <c r="D30" s="1">
+        <v>24000000</v>
+      </c>
+      <c r="E30" s="1">
+        <v>0</v>
+      </c>
+      <c r="F30" s="1">
+        <v>0</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="H30">
+        <v>0</v>
+      </c>
+      <c r="I30">
+        <v>22</v>
+      </c>
+      <c r="J30">
+        <v>11</v>
+      </c>
+      <c r="K30" s="1">
+        <f>ROUND((D30+E30+F30)*J30/I30,0)</f>
+        <v>12000000</v>
+      </c>
+      <c r="L30">
+        <v>0</v>
+      </c>
+      <c r="M30">
+        <v>0</v>
+      </c>
+      <c r="N30" s="1">
+        <f>ROUND((D30+E30)/I30/8*M30*L30,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O30" s="1">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="P30" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="1">
+        <f>K30+N30+O30+P30+AI30</f>
+        <v>28500000</v>
+      </c>
+      <c r="R30" s="1">
+        <f>ROUND((D30+E30)/I30/8*M30*MIN(L30,40),0)+O30+AI30</f>
+        <v>16500000</v>
+      </c>
+      <c r="S30" s="1">
+        <v>24000000</v>
+      </c>
+      <c r="T30" s="1">
+        <v>1920000</v>
+      </c>
+      <c r="U30" s="1">
+        <v>360000</v>
+      </c>
+      <c r="V30" s="1">
+        <v>240000</v>
+      </c>
+      <c r="W30" s="1">
+        <v>15500000</v>
+      </c>
+      <c r="X30" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y30" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z30" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA30" s="1">
+        <f>Q30-T30-U30-V30-Z30</f>
+        <v>25980000</v>
+      </c>
+      <c r="AB30" s="1">
+        <v>4200000</v>
+      </c>
+      <c r="AC30" s="1">
+        <v>720000</v>
+      </c>
+      <c r="AD30" s="1">
+        <v>240000</v>
+      </c>
+      <c r="AE30" s="1">
+        <v>480000</v>
+      </c>
+      <c r="AF30" s="1">
+        <f>Q30+AB30+AC30+AD30+AE30</f>
+        <v>34140000</v>
+      </c>
+      <c r="AG30" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="AH30" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI30" s="1">
+        <v>16500000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>136</v>
+      </c>
+      <c r="B31" t="s">
+        <v>137</v>
+      </c>
+      <c r="C31" t="s">
+        <v>37</v>
+      </c>
+      <c r="D31" s="1">
+        <v>15000000</v>
+      </c>
+      <c r="E31" s="1">
+        <v>0</v>
+      </c>
+      <c r="F31" s="1">
+        <v>0</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="H31">
+        <v>0</v>
+      </c>
+      <c r="I31">
+        <v>22</v>
+      </c>
+      <c r="J31">
+        <v>22</v>
+      </c>
+      <c r="K31" s="1">
+        <f>ROUND((D31+E31+F31)*J31/I31,0)</f>
+        <v>15000000</v>
+      </c>
+      <c r="L31">
+        <v>0</v>
+      </c>
+      <c r="M31">
+        <v>0</v>
+      </c>
+      <c r="N31" s="1">
+        <f>ROUND((D31+E31)/I31/8*M31*L31,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O31" s="1">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="P31" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="1">
+        <f>K31+N31+O31+P31+AI31</f>
+        <v>45000000</v>
+      </c>
+      <c r="R31" s="1">
+        <f>ROUND((D31+E31)/I31/8*M31*MIN(L31,40),0)+O31+AI31</f>
+        <v>30000000</v>
+      </c>
+      <c r="S31" s="1">
+        <v>15000000</v>
+      </c>
+      <c r="T31" s="1">
+        <v>1200000</v>
+      </c>
+      <c r="U31" s="1">
+        <v>225000</v>
+      </c>
+      <c r="V31" s="1">
+        <v>150000</v>
+      </c>
+      <c r="W31" s="1">
+        <v>15500000</v>
+      </c>
+      <c r="X31" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y31" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z31" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA31" s="1">
+        <f>Q31-T31-U31-V31-Z31</f>
+        <v>43425000</v>
+      </c>
+      <c r="AB31" s="1">
+        <v>2625000</v>
+      </c>
+      <c r="AC31" s="1">
+        <v>450000</v>
+      </c>
+      <c r="AD31" s="1">
+        <v>150000</v>
+      </c>
+      <c r="AE31" s="1">
+        <v>300000</v>
+      </c>
+      <c r="AF31" s="1">
+        <f>Q31+AB31+AC31+AD31+AE31</f>
+        <v>48525000</v>
+      </c>
+      <c r="AG31" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="AH31" t="s">
+        <v>140</v>
+      </c>
+      <c r="AI31" s="1">
+        <v>30000000</v>
       </c>
     </row>
   </sheetData>
@@ -4322,7 +4680,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -4333,16 +4691,16 @@
   <sheetData>
     <row r="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -4350,13 +4708,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -4367,10 +4725,10 @@
         <v>8</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -4378,13 +4736,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -4392,13 +4750,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -4406,13 +4764,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -4420,13 +4778,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>149</v>
+        <v>160</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -4437,10 +4795,10 @@
         <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>151</v>
+        <v>162</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>152</v>
+        <v>163</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -4448,13 +4806,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>153</v>
+        <v>164</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -4462,13 +4820,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>156</v>
+        <v>167</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>158</v>
+        <v>169</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -4476,13 +4834,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>18</v>
+        <v>170</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -4490,13 +4848,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>161</v>
+        <v>18</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -4504,13 +4862,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>164</v>
+        <v>175</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -4518,13 +4876,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>168</v>
+        <v>179</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>169</v>
+        <v>180</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -4532,13 +4890,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>172</v>
+        <v>183</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -4546,13 +4904,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>175</v>
+        <v>186</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -4560,13 +4918,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>176</v>
+        <v>187</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>177</v>
+        <v>188</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -4574,13 +4932,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -4588,13 +4946,27 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>184</v>
+        <v>195</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -4616,114 +4988,114 @@
   <sheetData>
     <row r="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>185</v>
+        <v>199</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>186</v>
+        <v>200</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>187</v>
+        <v>201</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>188</v>
+        <v>202</v>
       </c>
       <c r="B2" s="1">
         <v>5310000</v>
       </c>
       <c r="C2" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="D2" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>191</v>
+        <v>205</v>
       </c>
       <c r="B3" s="1">
         <v>2340000</v>
       </c>
       <c r="C3" t="s">
-        <v>192</v>
+        <v>206</v>
       </c>
       <c r="D3" t="s">
-        <v>193</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>191</v>
+        <v>205</v>
       </c>
       <c r="B4" s="1">
         <v>2530000</v>
       </c>
       <c r="C4" t="s">
-        <v>194</v>
+        <v>208</v>
       </c>
       <c r="D4" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>196</v>
+        <v>210</v>
       </c>
       <c r="B5" s="1">
         <v>46800000</v>
       </c>
       <c r="C5" t="s">
-        <v>192</v>
+        <v>206</v>
       </c>
       <c r="D5" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>197</v>
+        <v>211</v>
       </c>
       <c r="B6" s="1">
         <v>50600000</v>
       </c>
       <c r="C6" t="s">
-        <v>194</v>
+        <v>208</v>
       </c>
       <c r="D6" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>198</v>
+        <v>212</v>
       </c>
       <c r="B7" s="1">
         <v>106200000</v>
       </c>
       <c r="C7" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="D7" t="s">
-        <v>199</v>
+        <v>213</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>200</v>
+        <v>214</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>201</v>
+        <v>215</v>
       </c>
       <c r="C8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D8" t="s">
-        <v>202</v>
+        <v>216</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -4734,52 +5106,52 @@
         <v>15500000</v>
       </c>
       <c r="C9" t="s">
-        <v>203</v>
+        <v>217</v>
       </c>
       <c r="D9" t="s">
-        <v>204</v>
+        <v>218</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>205</v>
+        <v>219</v>
       </c>
       <c r="B10" s="1">
         <v>6200000</v>
       </c>
       <c r="C10" t="s">
-        <v>203</v>
+        <v>217</v>
       </c>
       <c r="D10" t="s">
-        <v>204</v>
+        <v>218</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>206</v>
+        <v>220</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>207</v>
+        <v>221</v>
       </c>
       <c r="C11" t="s">
-        <v>203</v>
+        <v>217</v>
       </c>
       <c r="D11" t="s">
-        <v>178</v>
+        <v>192</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>208</v>
+        <v>222</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="C12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D12" t="s">
-        <v>210</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -4799,50 +5171,50 @@
   <sheetData>
     <row r="1" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>211</v>
+        <v>225</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>212</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>213</v>
+        <v>227</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>214</v>
+        <v>228</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>215</v>
+        <v>229</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>216</v>
+        <v>230</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>217</v>
+        <v>231</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>218</v>
+        <v>232</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>219</v>
+        <v>233</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>221</v>
+        <v>235</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
     </row>
   </sheetData>

</xml_diff>